<commit_message>
shorten results and add combine header test case  to test_get_df_from_excel
</commit_message>
<xml_diff>
--- a/tests/data/mini-nodes-matrix.xlsx
+++ b/tests/data/mini-nodes-matrix.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="connectivity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="combined_header" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,4 +614,87 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mini_G nodes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>idx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>